<commit_message>
Updating all the markdown stuff. Specifically deleting the older draft documents and indicating, in the README that the subsequent descriptions of code and visualizations will be demonstrated on R pub.
</commit_message>
<xml_diff>
--- a/Immigration_Networks/IMF_GDPperCap_PPP.xlsx
+++ b/Immigration_Networks/IMF_GDPperCap_PPP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1402c53be3bc7c0d/Career/Professional_Portfolio/Network_Analysis/MigrationAmericas_NetworkAnalysis/Immigration_Networks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="8_{C96F5C29-266E-4132-A555-F268BF85E120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{268E3425-D303-4436-A535-2D9F5AA75EB5}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="8_{C96F5C29-266E-4132-A555-F268BF85E120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97366B62-D930-49B0-8BE0-DE083F5DD228}"/>
   <bookViews>
     <workbookView xWindow="1140" yWindow="620" windowWidth="14400" windowHeight="9460" xr2:uid="{F2A1BD2B-BB1E-4B80-91B5-E12871C060AC}"/>
   </bookViews>
@@ -17,6 +17,9 @@
     <sheet name="ReadMe" sheetId="3" r:id="rId2"/>
     <sheet name="RawDatafromIMF" sheetId="1" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'10yr Avgs'!$A$1:$F$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1078,6 +1081,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A9A9951-FC52-47F3-BCD4-9799BD194B1F}">
   <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="6" max="6" width="9" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -1141,345 +1147,350 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="1">
-        <v>6052.5846666666666</v>
+        <v>5933.3181666666669</v>
       </c>
       <c r="D4" s="1">
-        <v>7904.440333333333</v>
+        <v>9646.9521666666678</v>
       </c>
       <c r="E4" s="1">
-        <v>11717.686166666666</v>
+        <v>18237.170333333332</v>
       </c>
       <c r="F4" s="1">
-        <v>15141.388499999999</v>
+        <v>31433.994500000001</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
       <c r="C5" s="1">
-        <v>2877.2919999999999</v>
+        <v>4874.0135</v>
       </c>
       <c r="D5" s="1">
-        <v>4452.7008333333324</v>
+        <v>10141.271333333332</v>
       </c>
       <c r="E5" s="1">
-        <v>6512.7761666666665</v>
+        <v>17284.053166666668</v>
       </c>
       <c r="F5" s="1">
-        <v>10222.016333333333</v>
+        <v>24831.614833333329</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="C6" s="1">
-        <v>8274.7196666666659</v>
+        <v>6085.9823333333334</v>
       </c>
       <c r="D6" s="1">
-        <v>13035.211833333333</v>
+        <v>10102.238166666664</v>
       </c>
       <c r="E6" s="1">
-        <v>18919.113333333331</v>
+        <v>14523.258333333333</v>
       </c>
       <c r="F6" s="1">
-        <v>23293.706333333335</v>
+        <v>23367.039666666667</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="1">
-        <v>4304.7020000000002</v>
+        <v>8274.7196666666659</v>
       </c>
       <c r="D7" s="1">
-        <v>6552.7434999999996</v>
+        <v>13035.211833333333</v>
       </c>
       <c r="E7" s="1">
-        <v>9810.7588333333333</v>
+        <v>18919.113333333331</v>
       </c>
       <c r="F7" s="1">
-        <v>15075.876499999998</v>
+        <v>23293.706333333335</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="1">
-        <v>4874.0135</v>
+        <v>5332.3291666666673</v>
       </c>
       <c r="D8" s="1">
-        <v>10141.271333333332</v>
+        <v>8493.2379999999994</v>
       </c>
       <c r="E8" s="1">
-        <v>17284.053166666668</v>
+        <v>13820.530833333332</v>
       </c>
       <c r="F8" s="1">
-        <v>24831.614833333329</v>
+        <v>20744.308000000001</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
       </c>
       <c r="C9" s="1">
-        <v>2210.9920000000002</v>
+        <v>8442.2948333333334</v>
       </c>
       <c r="D9" s="1">
-        <v>2879.9226666666668</v>
+        <v>12258.029499999999</v>
       </c>
       <c r="E9" s="1">
-        <v>4255.2051666666666</v>
+        <v>16496.662500000002</v>
       </c>
       <c r="F9" s="1">
-        <v>5500.1798333333327</v>
+        <v>19989.367000000002</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
       </c>
       <c r="C10" s="1">
-        <v>5332.3291666666673</v>
+        <v>6052.5846666666666</v>
       </c>
       <c r="D10" s="1">
-        <v>8493.2379999999994</v>
+        <v>7904.440333333333</v>
       </c>
       <c r="E10" s="1">
-        <v>13820.530833333332</v>
+        <v>11717.686166666666</v>
       </c>
       <c r="F10" s="1">
-        <v>20744.308000000001</v>
+        <v>15141.388499999999</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="1">
-        <v>4073.0579999999995</v>
+        <v>4304.7020000000002</v>
       </c>
       <c r="D11" s="1">
-        <v>5569.2809999999999</v>
+        <v>6552.7434999999996</v>
       </c>
       <c r="E11" s="1">
-        <v>8163.3618333333334</v>
+        <v>9810.7588333333333</v>
       </c>
       <c r="F11" s="1">
-        <v>11720.807166666667</v>
+        <v>15075.876499999998</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="C12" s="1">
-        <v>2812.3748333333333</v>
+        <v>4723.9808333333331</v>
       </c>
       <c r="D12" s="1">
-        <v>4535.2830000000004</v>
+        <v>6720.3855000000003</v>
       </c>
       <c r="E12" s="1">
-        <v>6526.265166666667</v>
+        <v>9011.3396666666667</v>
       </c>
       <c r="F12" s="1">
-        <v>9051.7565000000013</v>
+        <v>14520.067999999999</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="C13" s="1">
-        <v>2333.6770000000001</v>
+        <v>3659.6264999999999</v>
       </c>
       <c r="D13" s="1">
-        <v>2729.7270000000003</v>
+        <v>4619.8575000000001</v>
       </c>
       <c r="E13" s="1">
-        <v>4006.8496666666665</v>
+        <v>8046.7833333333328</v>
       </c>
       <c r="F13" s="1">
-        <v>5939.0941666666668</v>
+        <v>13283.342666666666</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
       </c>
       <c r="C14" s="1">
-        <v>5933.3181666666669</v>
+        <v>4073.0579999999995</v>
       </c>
       <c r="D14" s="1">
-        <v>9646.9521666666678</v>
+        <v>5569.2809999999999</v>
       </c>
       <c r="E14" s="1">
-        <v>18237.170333333332</v>
+        <v>8163.3618333333334</v>
       </c>
       <c r="F14" s="1">
-        <v>31433.994500000001</v>
+        <v>11720.807166666667</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>51</v>
       </c>
       <c r="C15" s="1">
-        <v>3660.1101666666668</v>
+        <v>9446.4575000000004</v>
       </c>
       <c r="D15" s="1">
-        <v>5156.2986666666666</v>
+        <v>11738.970833333335</v>
       </c>
       <c r="E15" s="1">
-        <v>7222.6699999999992</v>
+        <v>16174.63</v>
       </c>
       <c r="F15" s="1">
-        <v>9934.4711666666644</v>
+        <v>11313.420166666669</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B16" t="s">
         <v>11</v>
       </c>
       <c r="C16" s="1">
-        <v>8442.2948333333334</v>
+        <v>2877.2919999999999</v>
       </c>
       <c r="D16" s="1">
-        <v>12258.029499999999</v>
+        <v>4452.7008333333324</v>
       </c>
       <c r="E16" s="1">
-        <v>16496.662500000002</v>
+        <v>6512.7761666666665</v>
       </c>
       <c r="F16" s="1">
-        <v>19989.367000000002</v>
+        <v>10222.016333333333</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s">
-        <v>51</v>
+        <v>11</v>
       </c>
       <c r="C17" s="1">
-        <v>9446.4575000000004</v>
+        <v>3660.1101666666668</v>
       </c>
       <c r="D17" s="1">
-        <v>11738.970833333335</v>
+        <v>5156.2986666666666</v>
       </c>
       <c r="E17" s="1">
-        <v>16174.63</v>
+        <v>7222.6699999999992</v>
       </c>
       <c r="F17" s="1">
-        <v>11313.420166666669</v>
+        <v>9934.4711666666644</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B18" t="s">
-        <v>52</v>
+        <v>11</v>
       </c>
       <c r="C18" s="1">
-        <v>6085.9823333333334</v>
+        <v>2812.3748333333333</v>
       </c>
       <c r="D18" s="1">
-        <v>10102.238166666664</v>
+        <v>4535.2830000000004</v>
       </c>
       <c r="E18" s="1">
-        <v>14523.258333333333</v>
+        <v>6526.265166666667</v>
       </c>
       <c r="F18" s="1">
-        <v>23367.039666666667</v>
+        <v>9051.7565000000013</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="C19" s="1">
-        <v>4723.9808333333331</v>
+        <v>2333.6770000000001</v>
       </c>
       <c r="D19" s="1">
-        <v>6720.3855000000003</v>
+        <v>2729.7270000000003</v>
       </c>
       <c r="E19" s="1">
-        <v>9011.3396666666667</v>
+        <v>4006.8496666666665</v>
       </c>
       <c r="F19" s="1">
-        <v>14520.067999999999</v>
+        <v>5939.0941666666668</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="C20" s="1">
-        <v>3659.6264999999999</v>
+        <v>2210.9920000000002</v>
       </c>
       <c r="D20" s="1">
-        <v>4619.8575000000001</v>
+        <v>2879.9226666666668</v>
       </c>
       <c r="E20" s="1">
-        <v>8046.7833333333328</v>
+        <v>4255.2051666666666</v>
       </c>
       <c r="F20" s="1">
-        <v>13283.342666666666</v>
+        <v>5500.1798333333327</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F1" xr:uid="{2A9A9951-FC52-47F3-BCD4-9799BD194B1F}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F20">
+      <sortCondition descending="1" ref="F1"/>
+    </sortState>
+  </autoFilter>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>